<commit_message>
Add 2026 subscriptions and prevent duplicate uploads
Make the subscription import process idempotent by checking for existing member-year combinations and update the UI to display skipped records. Also adds 2026 subscription data to the provided Excel file.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b7ec80f7-5a29-4121-9a7a-a68917e6e326
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b2ddac2e-7a01-4d47-8b76-b3710659e0a6
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f5e3303d-597c-4653-a566-198199961662/b7ec80f7-5a29-4121-9a7a-a68917e6e326/kALypKz
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/اشتراكات-تجريبية-SCVA.xlsx
+++ b/اشتراكات-تجريبية-SCVA.xlsx
@@ -397,15 +397,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G290"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4801,9 +4801,2286 @@
         <v/>
       </c>
     </row>
+    <row r="192">
+      <c r="A192">
+        <v>1</v>
+      </c>
+      <c r="B192" t="str">
+        <v>حسن</v>
+      </c>
+      <c r="C192" t="str">
+        <v>الشامي</v>
+      </c>
+      <c r="D192">
+        <v>2026</v>
+      </c>
+      <c r="E192">
+        <v>200000</v>
+      </c>
+      <c r="F192" t="str">
+        <v>2026-07-18</v>
+      </c>
+      <c r="G192" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193">
+        <v>2</v>
+      </c>
+      <c r="B193" t="str">
+        <v>ماجد</v>
+      </c>
+      <c r="C193" t="str">
+        <v>التميمي</v>
+      </c>
+      <c r="D193">
+        <v>2026</v>
+      </c>
+      <c r="E193">
+        <v>250000</v>
+      </c>
+      <c r="F193" t="str">
+        <v>2026-06-21</v>
+      </c>
+      <c r="G193" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194">
+        <v>3</v>
+      </c>
+      <c r="B194" t="str">
+        <v>وائل</v>
+      </c>
+      <c r="C194" t="str">
+        <v>المغربي</v>
+      </c>
+      <c r="D194">
+        <v>2026</v>
+      </c>
+      <c r="E194">
+        <v>200000</v>
+      </c>
+      <c r="F194" t="str">
+        <v>2026-02-09</v>
+      </c>
+      <c r="G194" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195">
+        <v>4</v>
+      </c>
+      <c r="B195" t="str">
+        <v>فيصل</v>
+      </c>
+      <c r="C195" t="str">
+        <v>السليمان</v>
+      </c>
+      <c r="D195">
+        <v>2026</v>
+      </c>
+      <c r="E195">
+        <v>300000</v>
+      </c>
+      <c r="F195" t="str">
+        <v>2026-11-26</v>
+      </c>
+      <c r="G195" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>5</v>
+      </c>
+      <c r="B196" t="str">
+        <v>غسان</v>
+      </c>
+      <c r="C196" t="str">
+        <v>الجراح</v>
+      </c>
+      <c r="D196">
+        <v>2026</v>
+      </c>
+      <c r="E196">
+        <v>200000</v>
+      </c>
+      <c r="F196" t="str">
+        <v>2026-10-11</v>
+      </c>
+      <c r="G196" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>6</v>
+      </c>
+      <c r="B197" t="str">
+        <v>نزار</v>
+      </c>
+      <c r="C197" t="str">
+        <v>الكلاس</v>
+      </c>
+      <c r="D197">
+        <v>2026</v>
+      </c>
+      <c r="E197">
+        <v>200000</v>
+      </c>
+      <c r="F197" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="G197" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>7</v>
+      </c>
+      <c r="B198" t="str">
+        <v>لؤي</v>
+      </c>
+      <c r="C198" t="str">
+        <v>العاصي</v>
+      </c>
+      <c r="D198">
+        <v>2026</v>
+      </c>
+      <c r="E198">
+        <v>200000</v>
+      </c>
+      <c r="F198" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="G198" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>8</v>
+      </c>
+      <c r="B199" t="str">
+        <v>نزار</v>
+      </c>
+      <c r="C199" t="str">
+        <v>العاصي</v>
+      </c>
+      <c r="D199">
+        <v>2026</v>
+      </c>
+      <c r="E199">
+        <v>200000</v>
+      </c>
+      <c r="F199" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="G199" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>9</v>
+      </c>
+      <c r="B200" t="str">
+        <v>شادي</v>
+      </c>
+      <c r="C200" t="str">
+        <v>الجسر</v>
+      </c>
+      <c r="D200">
+        <v>2026</v>
+      </c>
+      <c r="E200">
+        <v>250000</v>
+      </c>
+      <c r="F200" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G200" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>10</v>
+      </c>
+      <c r="B201" t="str">
+        <v>إبراهيم</v>
+      </c>
+      <c r="C201" t="str">
+        <v>العمر</v>
+      </c>
+      <c r="D201">
+        <v>2026</v>
+      </c>
+      <c r="E201">
+        <v>200000</v>
+      </c>
+      <c r="F201" t="str">
+        <v>2026-10-09</v>
+      </c>
+      <c r="G201" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202">
+        <v>11</v>
+      </c>
+      <c r="B202" t="str">
+        <v>علي</v>
+      </c>
+      <c r="C202" t="str">
+        <v>الحمصي</v>
+      </c>
+      <c r="D202">
+        <v>2026</v>
+      </c>
+      <c r="E202">
+        <v>300000</v>
+      </c>
+      <c r="F202" t="str">
+        <v>2026-11-11</v>
+      </c>
+      <c r="G202" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203">
+        <v>12</v>
+      </c>
+      <c r="B203" t="str">
+        <v>باسم</v>
+      </c>
+      <c r="C203" t="str">
+        <v>الكلاس</v>
+      </c>
+      <c r="D203">
+        <v>2026</v>
+      </c>
+      <c r="E203">
+        <v>200000</v>
+      </c>
+      <c r="F203" t="str">
+        <v>2026-11-09</v>
+      </c>
+      <c r="G203" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204">
+        <v>13</v>
+      </c>
+      <c r="B204" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C204" t="str">
+        <v>الجراح</v>
+      </c>
+      <c r="D204">
+        <v>2026</v>
+      </c>
+      <c r="E204">
+        <v>200000</v>
+      </c>
+      <c r="F204" t="str">
+        <v>2026-02-01</v>
+      </c>
+      <c r="G204" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205">
+        <v>14</v>
+      </c>
+      <c r="B205" t="str">
+        <v>يوسف</v>
+      </c>
+      <c r="C205" t="str">
+        <v>القاسم</v>
+      </c>
+      <c r="D205">
+        <v>2026</v>
+      </c>
+      <c r="E205">
+        <v>200000</v>
+      </c>
+      <c r="F205" t="str">
+        <v>2026-11-05</v>
+      </c>
+      <c r="G205" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206">
+        <v>15</v>
+      </c>
+      <c r="B206" t="str">
+        <v>وليد</v>
+      </c>
+      <c r="C206" t="str">
+        <v>الحلبي</v>
+      </c>
+      <c r="D206">
+        <v>2026</v>
+      </c>
+      <c r="E206">
+        <v>200000</v>
+      </c>
+      <c r="F206" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="G206" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207">
+        <v>16</v>
+      </c>
+      <c r="B207" t="str">
+        <v>علي</v>
+      </c>
+      <c r="C207" t="str">
+        <v>المهايني</v>
+      </c>
+      <c r="D207">
+        <v>2026</v>
+      </c>
+      <c r="E207">
+        <v>250000</v>
+      </c>
+      <c r="F207" t="str">
+        <v>2026-07-19</v>
+      </c>
+      <c r="G207" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208">
+        <v>17</v>
+      </c>
+      <c r="B208" t="str">
+        <v>سعد</v>
+      </c>
+      <c r="C208" t="str">
+        <v>اليوسف</v>
+      </c>
+      <c r="D208">
+        <v>2026</v>
+      </c>
+      <c r="E208">
+        <v>200000</v>
+      </c>
+      <c r="F208" t="str">
+        <v>2026-02-22</v>
+      </c>
+      <c r="G208" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209">
+        <v>18</v>
+      </c>
+      <c r="B209" t="str">
+        <v>نزار</v>
+      </c>
+      <c r="C209" t="str">
+        <v>الحسين</v>
+      </c>
+      <c r="D209">
+        <v>2026</v>
+      </c>
+      <c r="E209">
+        <v>300000</v>
+      </c>
+      <c r="F209" t="str">
+        <v>2026-07-08</v>
+      </c>
+      <c r="G209" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210">
+        <v>19</v>
+      </c>
+      <c r="B210" t="str">
+        <v>وائل</v>
+      </c>
+      <c r="C210" t="str">
+        <v>الطيب</v>
+      </c>
+      <c r="D210">
+        <v>2026</v>
+      </c>
+      <c r="E210">
+        <v>200000</v>
+      </c>
+      <c r="F210" t="str">
+        <v>2026-11-20</v>
+      </c>
+      <c r="G210" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211">
+        <v>20</v>
+      </c>
+      <c r="B211" t="str">
+        <v>حسن</v>
+      </c>
+      <c r="C211" t="str">
+        <v>القباني</v>
+      </c>
+      <c r="D211">
+        <v>2026</v>
+      </c>
+      <c r="E211">
+        <v>200000</v>
+      </c>
+      <c r="F211" t="str">
+        <v>2026-02-22</v>
+      </c>
+      <c r="G211" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212">
+        <v>21</v>
+      </c>
+      <c r="B212" t="str">
+        <v>حسن</v>
+      </c>
+      <c r="C212" t="str">
+        <v>الدندشي</v>
+      </c>
+      <c r="D212">
+        <v>2026</v>
+      </c>
+      <c r="E212">
+        <v>200000</v>
+      </c>
+      <c r="F212" t="str">
+        <v>2026-11-21</v>
+      </c>
+      <c r="G212" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213">
+        <v>22</v>
+      </c>
+      <c r="B213" t="str">
+        <v>فيصل</v>
+      </c>
+      <c r="C213" t="str">
+        <v>القباني</v>
+      </c>
+      <c r="D213">
+        <v>2026</v>
+      </c>
+      <c r="E213">
+        <v>200000</v>
+      </c>
+      <c r="F213" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="G213" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214">
+        <v>23</v>
+      </c>
+      <c r="B214" t="str">
+        <v>عماد</v>
+      </c>
+      <c r="C214" t="str">
+        <v>الهاشم</v>
+      </c>
+      <c r="D214">
+        <v>2026</v>
+      </c>
+      <c r="E214">
+        <v>250000</v>
+      </c>
+      <c r="F214" t="str">
+        <v>2026-11-25</v>
+      </c>
+      <c r="G214" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215">
+        <v>24</v>
+      </c>
+      <c r="B215" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C215" t="str">
+        <v>الدمشقي</v>
+      </c>
+      <c r="D215">
+        <v>2026</v>
+      </c>
+      <c r="E215">
+        <v>200000</v>
+      </c>
+      <c r="F215" t="str">
+        <v>2026-10-08</v>
+      </c>
+      <c r="G215" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216">
+        <v>25</v>
+      </c>
+      <c r="B216" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C216" t="str">
+        <v>الكيلاني</v>
+      </c>
+      <c r="D216">
+        <v>2026</v>
+      </c>
+      <c r="E216">
+        <v>300000</v>
+      </c>
+      <c r="F216" t="str">
+        <v>2026-01-15</v>
+      </c>
+      <c r="G216" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217">
+        <v>26</v>
+      </c>
+      <c r="B217" t="str">
+        <v>نضال</v>
+      </c>
+      <c r="C217" t="str">
+        <v>الدباغ</v>
+      </c>
+      <c r="D217">
+        <v>2026</v>
+      </c>
+      <c r="E217">
+        <v>200000</v>
+      </c>
+      <c r="F217" t="str">
+        <v>2026-08-04</v>
+      </c>
+      <c r="G217" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218">
+        <v>27</v>
+      </c>
+      <c r="B218" t="str">
+        <v>يوسف</v>
+      </c>
+      <c r="C218" t="str">
+        <v>الشريف</v>
+      </c>
+      <c r="D218">
+        <v>2026</v>
+      </c>
+      <c r="E218">
+        <v>200000</v>
+      </c>
+      <c r="F218" t="str">
+        <v>2026-06-07</v>
+      </c>
+      <c r="G218" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219">
+        <v>28</v>
+      </c>
+      <c r="B219" t="str">
+        <v>رامي</v>
+      </c>
+      <c r="C219" t="str">
+        <v>الشامي</v>
+      </c>
+      <c r="D219">
+        <v>2026</v>
+      </c>
+      <c r="E219">
+        <v>200000</v>
+      </c>
+      <c r="F219" t="str">
+        <v>2026-11-03</v>
+      </c>
+      <c r="G219" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220">
+        <v>29</v>
+      </c>
+      <c r="B220" t="str">
+        <v>جمال</v>
+      </c>
+      <c r="C220" t="str">
+        <v>المصري</v>
+      </c>
+      <c r="D220">
+        <v>2026</v>
+      </c>
+      <c r="E220">
+        <v>200000</v>
+      </c>
+      <c r="F220" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="G220" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221">
+        <v>30</v>
+      </c>
+      <c r="B221" t="str">
+        <v>كمال</v>
+      </c>
+      <c r="C221" t="str">
+        <v>الشريف</v>
+      </c>
+      <c r="D221">
+        <v>2026</v>
+      </c>
+      <c r="E221">
+        <v>250000</v>
+      </c>
+      <c r="F221" t="str">
+        <v>2026-06-06</v>
+      </c>
+      <c r="G221" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222">
+        <v>31</v>
+      </c>
+      <c r="B222" t="str">
+        <v>سعد</v>
+      </c>
+      <c r="C222" t="str">
+        <v>الدمشقي</v>
+      </c>
+      <c r="D222">
+        <v>2026</v>
+      </c>
+      <c r="E222">
+        <v>200000</v>
+      </c>
+      <c r="F222" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="G222" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223">
+        <v>32</v>
+      </c>
+      <c r="B223" t="str">
+        <v>علي</v>
+      </c>
+      <c r="C223" t="str">
+        <v>الهاشم</v>
+      </c>
+      <c r="D223">
+        <v>2026</v>
+      </c>
+      <c r="E223">
+        <v>300000</v>
+      </c>
+      <c r="F223" t="str">
+        <v>2026-07-21</v>
+      </c>
+      <c r="G223" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224">
+        <v>33</v>
+      </c>
+      <c r="B224" t="str">
+        <v>لؤي</v>
+      </c>
+      <c r="C224" t="str">
+        <v>الزعيم</v>
+      </c>
+      <c r="D224">
+        <v>2026</v>
+      </c>
+      <c r="E224">
+        <v>200000</v>
+      </c>
+      <c r="F224" t="str">
+        <v>2026-05-17</v>
+      </c>
+      <c r="G224" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225">
+        <v>34</v>
+      </c>
+      <c r="B225" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C225" t="str">
+        <v>الحسن</v>
+      </c>
+      <c r="D225">
+        <v>2026</v>
+      </c>
+      <c r="E225">
+        <v>200000</v>
+      </c>
+      <c r="F225" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="G225" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226">
+        <v>35</v>
+      </c>
+      <c r="B226" t="str">
+        <v>عماد</v>
+      </c>
+      <c r="C226" t="str">
+        <v>العلي</v>
+      </c>
+      <c r="D226">
+        <v>2026</v>
+      </c>
+      <c r="E226">
+        <v>200000</v>
+      </c>
+      <c r="F226" t="str">
+        <v>2026-11-28</v>
+      </c>
+      <c r="G226" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227">
+        <v>36</v>
+      </c>
+      <c r="B227" t="str">
+        <v>نبيل</v>
+      </c>
+      <c r="C227" t="str">
+        <v>العظمة</v>
+      </c>
+      <c r="D227">
+        <v>2026</v>
+      </c>
+      <c r="E227">
+        <v>200000</v>
+      </c>
+      <c r="F227" t="str">
+        <v>2026-05-09</v>
+      </c>
+      <c r="G227" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228">
+        <v>37</v>
+      </c>
+      <c r="B228" t="str">
+        <v>فادي</v>
+      </c>
+      <c r="C228" t="str">
+        <v>الدباغ</v>
+      </c>
+      <c r="D228">
+        <v>2026</v>
+      </c>
+      <c r="E228">
+        <v>250000</v>
+      </c>
+      <c r="F228" t="str">
+        <v>2026-03-12</v>
+      </c>
+      <c r="G228" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229">
+        <v>38</v>
+      </c>
+      <c r="B229" t="str">
+        <v>عماد</v>
+      </c>
+      <c r="C229" t="str">
+        <v>الدمشقي</v>
+      </c>
+      <c r="D229">
+        <v>2026</v>
+      </c>
+      <c r="E229">
+        <v>200000</v>
+      </c>
+      <c r="F229" t="str">
+        <v>2026-02-26</v>
+      </c>
+      <c r="G229" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230">
+        <v>39</v>
+      </c>
+      <c r="B230" t="str">
+        <v>فادي</v>
+      </c>
+      <c r="C230" t="str">
+        <v>الكلاس</v>
+      </c>
+      <c r="D230">
+        <v>2026</v>
+      </c>
+      <c r="E230">
+        <v>300000</v>
+      </c>
+      <c r="F230" t="str">
+        <v>2026-01-24</v>
+      </c>
+      <c r="G230" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231">
+        <v>40</v>
+      </c>
+      <c r="B231" t="str">
+        <v>سامر</v>
+      </c>
+      <c r="C231" t="str">
+        <v>المغربي</v>
+      </c>
+      <c r="D231">
+        <v>2026</v>
+      </c>
+      <c r="E231">
+        <v>200000</v>
+      </c>
+      <c r="F231" t="str">
+        <v>2026-01-23</v>
+      </c>
+      <c r="G231" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232">
+        <v>41</v>
+      </c>
+      <c r="B232" t="str">
+        <v>باسم</v>
+      </c>
+      <c r="C232" t="str">
+        <v>القاسم</v>
+      </c>
+      <c r="D232">
+        <v>2026</v>
+      </c>
+      <c r="E232">
+        <v>200000</v>
+      </c>
+      <c r="F232" t="str">
+        <v>2026-02-27</v>
+      </c>
+      <c r="G232" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233">
+        <v>42</v>
+      </c>
+      <c r="B233" t="str">
+        <v>زياد</v>
+      </c>
+      <c r="C233" t="str">
+        <v>السليمان</v>
+      </c>
+      <c r="D233">
+        <v>2026</v>
+      </c>
+      <c r="E233">
+        <v>200000</v>
+      </c>
+      <c r="F233" t="str">
+        <v>2026-10-07</v>
+      </c>
+      <c r="G233" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234">
+        <v>43</v>
+      </c>
+      <c r="B234" t="str">
+        <v>خالد</v>
+      </c>
+      <c r="C234" t="str">
+        <v>الخطيب</v>
+      </c>
+      <c r="D234">
+        <v>2026</v>
+      </c>
+      <c r="E234">
+        <v>200000</v>
+      </c>
+      <c r="F234" t="str">
+        <v>2026-05-21</v>
+      </c>
+      <c r="G234" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235">
+        <v>44</v>
+      </c>
+      <c r="B235" t="str">
+        <v>أحمد</v>
+      </c>
+      <c r="C235" t="str">
+        <v>العظمة</v>
+      </c>
+      <c r="D235">
+        <v>2026</v>
+      </c>
+      <c r="E235">
+        <v>250000</v>
+      </c>
+      <c r="F235" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="G235" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236">
+        <v>45</v>
+      </c>
+      <c r="B236" t="str">
+        <v>عماد</v>
+      </c>
+      <c r="C236" t="str">
+        <v>البني</v>
+      </c>
+      <c r="D236">
+        <v>2026</v>
+      </c>
+      <c r="E236">
+        <v>200000</v>
+      </c>
+      <c r="F236" t="str">
+        <v>2026-02-11</v>
+      </c>
+      <c r="G236" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237">
+        <v>46</v>
+      </c>
+      <c r="B237" t="str">
+        <v>جمال</v>
+      </c>
+      <c r="C237" t="str">
+        <v>الكلاس</v>
+      </c>
+      <c r="D237">
+        <v>2026</v>
+      </c>
+      <c r="E237">
+        <v>300000</v>
+      </c>
+      <c r="F237" t="str">
+        <v>2026-01-14</v>
+      </c>
+      <c r="G237" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238">
+        <v>47</v>
+      </c>
+      <c r="B238" t="str">
+        <v>فيصل</v>
+      </c>
+      <c r="C238" t="str">
+        <v>المحمد</v>
+      </c>
+      <c r="D238">
+        <v>2026</v>
+      </c>
+      <c r="E238">
+        <v>200000</v>
+      </c>
+      <c r="F238" t="str">
+        <v>2026-08-08</v>
+      </c>
+      <c r="G238" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239">
+        <v>48</v>
+      </c>
+      <c r="B239" t="str">
+        <v>لؤي</v>
+      </c>
+      <c r="C239" t="str">
+        <v>الشامي</v>
+      </c>
+      <c r="D239">
+        <v>2026</v>
+      </c>
+      <c r="E239">
+        <v>200000</v>
+      </c>
+      <c r="F239" t="str">
+        <v>2026-11-10</v>
+      </c>
+      <c r="G239" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240">
+        <v>49</v>
+      </c>
+      <c r="B240" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C240" t="str">
+        <v>الحمصي</v>
+      </c>
+      <c r="D240">
+        <v>2026</v>
+      </c>
+      <c r="E240">
+        <v>200000</v>
+      </c>
+      <c r="F240" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="G240" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241">
+        <v>50</v>
+      </c>
+      <c r="B241" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C241" t="str">
+        <v>الجراح</v>
+      </c>
+      <c r="D241">
+        <v>2026</v>
+      </c>
+      <c r="E241">
+        <v>200000</v>
+      </c>
+      <c r="F241" t="str">
+        <v>2026-07-10</v>
+      </c>
+      <c r="G241" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242">
+        <v>51</v>
+      </c>
+      <c r="B242" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C242" t="str">
+        <v>البني</v>
+      </c>
+      <c r="D242">
+        <v>2026</v>
+      </c>
+      <c r="E242">
+        <v>250000</v>
+      </c>
+      <c r="F242" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="G242" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243">
+        <v>52</v>
+      </c>
+      <c r="B243" t="str">
+        <v>فادي</v>
+      </c>
+      <c r="C243" t="str">
+        <v>الزين</v>
+      </c>
+      <c r="D243">
+        <v>2026</v>
+      </c>
+      <c r="E243">
+        <v>200000</v>
+      </c>
+      <c r="F243" t="str">
+        <v>2026-03-03</v>
+      </c>
+      <c r="G243" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244">
+        <v>53</v>
+      </c>
+      <c r="B244" t="str">
+        <v>غسان</v>
+      </c>
+      <c r="C244" t="str">
+        <v>السيد</v>
+      </c>
+      <c r="D244">
+        <v>2026</v>
+      </c>
+      <c r="E244">
+        <v>300000</v>
+      </c>
+      <c r="F244" t="str">
+        <v>2026-05-27</v>
+      </c>
+      <c r="G244" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245">
+        <v>54</v>
+      </c>
+      <c r="B245" t="str">
+        <v>محمد</v>
+      </c>
+      <c r="C245" t="str">
+        <v>الأحمد</v>
+      </c>
+      <c r="D245">
+        <v>2026</v>
+      </c>
+      <c r="E245">
+        <v>200000</v>
+      </c>
+      <c r="F245" t="str">
+        <v>2026-03-02</v>
+      </c>
+      <c r="G245" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246">
+        <v>55</v>
+      </c>
+      <c r="B246" t="str">
+        <v>علي</v>
+      </c>
+      <c r="C246" t="str">
+        <v>القباني</v>
+      </c>
+      <c r="D246">
+        <v>2026</v>
+      </c>
+      <c r="E246">
+        <v>200000</v>
+      </c>
+      <c r="F246" t="str">
+        <v>2026-01-15</v>
+      </c>
+      <c r="G246" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247">
+        <v>56</v>
+      </c>
+      <c r="B247" t="str">
+        <v>نبيل</v>
+      </c>
+      <c r="C247" t="str">
+        <v>البدران</v>
+      </c>
+      <c r="D247">
+        <v>2026</v>
+      </c>
+      <c r="E247">
+        <v>200000</v>
+      </c>
+      <c r="F247" t="str">
+        <v>2026-10-09</v>
+      </c>
+      <c r="G247" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248">
+        <v>57</v>
+      </c>
+      <c r="B248" t="str">
+        <v>سعد</v>
+      </c>
+      <c r="C248" t="str">
+        <v>الجسر</v>
+      </c>
+      <c r="D248">
+        <v>2026</v>
+      </c>
+      <c r="E248">
+        <v>200000</v>
+      </c>
+      <c r="F248" t="str">
+        <v>2026-02-09</v>
+      </c>
+      <c r="G248" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249">
+        <v>58</v>
+      </c>
+      <c r="B249" t="str">
+        <v>كمال</v>
+      </c>
+      <c r="C249" t="str">
+        <v>المغربي</v>
+      </c>
+      <c r="D249">
+        <v>2026</v>
+      </c>
+      <c r="E249">
+        <v>250000</v>
+      </c>
+      <c r="F249" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="G249" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250">
+        <v>59</v>
+      </c>
+      <c r="B250" t="str">
+        <v>محمد</v>
+      </c>
+      <c r="C250" t="str">
+        <v>العلي</v>
+      </c>
+      <c r="D250">
+        <v>2026</v>
+      </c>
+      <c r="E250">
+        <v>200000</v>
+      </c>
+      <c r="F250" t="str">
+        <v>2026-04-06</v>
+      </c>
+      <c r="G250" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251">
+        <v>60</v>
+      </c>
+      <c r="B251" t="str">
+        <v>طارق</v>
+      </c>
+      <c r="C251" t="str">
+        <v>البني</v>
+      </c>
+      <c r="D251">
+        <v>2026</v>
+      </c>
+      <c r="E251">
+        <v>300000</v>
+      </c>
+      <c r="F251" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="G251" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252">
+        <v>61</v>
+      </c>
+      <c r="B252" t="str">
+        <v>حسين</v>
+      </c>
+      <c r="C252" t="str">
+        <v>المهايني</v>
+      </c>
+      <c r="D252">
+        <v>2026</v>
+      </c>
+      <c r="E252">
+        <v>200000</v>
+      </c>
+      <c r="F252" t="str">
+        <v>2026-07-14</v>
+      </c>
+      <c r="G252" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253">
+        <v>62</v>
+      </c>
+      <c r="B253" t="str">
+        <v>فيصل</v>
+      </c>
+      <c r="C253" t="str">
+        <v>الشامي</v>
+      </c>
+      <c r="D253">
+        <v>2026</v>
+      </c>
+      <c r="E253">
+        <v>200000</v>
+      </c>
+      <c r="F253" t="str">
+        <v>2026-07-18</v>
+      </c>
+      <c r="G253" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254">
+        <v>63</v>
+      </c>
+      <c r="B254" t="str">
+        <v>كمال</v>
+      </c>
+      <c r="C254" t="str">
+        <v>القباني</v>
+      </c>
+      <c r="D254">
+        <v>2026</v>
+      </c>
+      <c r="E254">
+        <v>200000</v>
+      </c>
+      <c r="F254" t="str">
+        <v>2026-03-19</v>
+      </c>
+      <c r="G254" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255">
+        <v>64</v>
+      </c>
+      <c r="B255" t="str">
+        <v>ماجد</v>
+      </c>
+      <c r="C255" t="str">
+        <v>الزين</v>
+      </c>
+      <c r="D255">
+        <v>2026</v>
+      </c>
+      <c r="E255">
+        <v>200000</v>
+      </c>
+      <c r="F255" t="str">
+        <v>2026-07-20</v>
+      </c>
+      <c r="G255" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256">
+        <v>65</v>
+      </c>
+      <c r="B256" t="str">
+        <v>وليد</v>
+      </c>
+      <c r="C256" t="str">
+        <v>العلي</v>
+      </c>
+      <c r="D256">
+        <v>2026</v>
+      </c>
+      <c r="E256">
+        <v>250000</v>
+      </c>
+      <c r="F256" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="G256" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257">
+        <v>66</v>
+      </c>
+      <c r="B257" t="str">
+        <v>يوسف</v>
+      </c>
+      <c r="C257" t="str">
+        <v>المهايني</v>
+      </c>
+      <c r="D257">
+        <v>2026</v>
+      </c>
+      <c r="E257">
+        <v>200000</v>
+      </c>
+      <c r="F257" t="str">
+        <v>2026-03-18</v>
+      </c>
+      <c r="G257" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258">
+        <v>67</v>
+      </c>
+      <c r="B258" t="str">
+        <v>لؤي</v>
+      </c>
+      <c r="C258" t="str">
+        <v>العظمة</v>
+      </c>
+      <c r="D258">
+        <v>2026</v>
+      </c>
+      <c r="E258">
+        <v>300000</v>
+      </c>
+      <c r="F258" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="G258" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259">
+        <v>68</v>
+      </c>
+      <c r="B259" t="str">
+        <v>عماد</v>
+      </c>
+      <c r="C259" t="str">
+        <v>القاسم</v>
+      </c>
+      <c r="D259">
+        <v>2026</v>
+      </c>
+      <c r="E259">
+        <v>200000</v>
+      </c>
+      <c r="F259" t="str">
+        <v>2026-01-17</v>
+      </c>
+      <c r="G259" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260">
+        <v>69</v>
+      </c>
+      <c r="B260" t="str">
+        <v>غسان</v>
+      </c>
+      <c r="C260" t="str">
+        <v>الحسين</v>
+      </c>
+      <c r="D260">
+        <v>2026</v>
+      </c>
+      <c r="E260">
+        <v>200000</v>
+      </c>
+      <c r="F260" t="str">
+        <v>2026-11-19</v>
+      </c>
+      <c r="G260" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261">
+        <v>70</v>
+      </c>
+      <c r="B261" t="str">
+        <v>محمد</v>
+      </c>
+      <c r="C261" t="str">
+        <v>الحلبي</v>
+      </c>
+      <c r="D261">
+        <v>2026</v>
+      </c>
+      <c r="E261">
+        <v>200000</v>
+      </c>
+      <c r="F261" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="G261" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262">
+        <v>71</v>
+      </c>
+      <c r="B262" t="str">
+        <v>إبراهيم</v>
+      </c>
+      <c r="C262" t="str">
+        <v>البدران</v>
+      </c>
+      <c r="D262">
+        <v>2026</v>
+      </c>
+      <c r="E262">
+        <v>200000</v>
+      </c>
+      <c r="F262" t="str">
+        <v>2026-07-06</v>
+      </c>
+      <c r="G262" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263">
+        <v>72</v>
+      </c>
+      <c r="B263" t="str">
+        <v>وليد</v>
+      </c>
+      <c r="C263" t="str">
+        <v>الدمشقي</v>
+      </c>
+      <c r="D263">
+        <v>2026</v>
+      </c>
+      <c r="E263">
+        <v>250000</v>
+      </c>
+      <c r="F263" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="G263" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264">
+        <v>73</v>
+      </c>
+      <c r="B264" t="str">
+        <v>باسم</v>
+      </c>
+      <c r="C264" t="str">
+        <v>المغربي</v>
+      </c>
+      <c r="D264">
+        <v>2026</v>
+      </c>
+      <c r="E264">
+        <v>200000</v>
+      </c>
+      <c r="F264" t="str">
+        <v>2026-05-25</v>
+      </c>
+      <c r="G264" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265">
+        <v>74</v>
+      </c>
+      <c r="B265" t="str">
+        <v>كمال</v>
+      </c>
+      <c r="C265" t="str">
+        <v>الخطيب</v>
+      </c>
+      <c r="D265">
+        <v>2026</v>
+      </c>
+      <c r="E265">
+        <v>300000</v>
+      </c>
+      <c r="F265" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="G265" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266">
+        <v>75</v>
+      </c>
+      <c r="B266" t="str">
+        <v>سمر</v>
+      </c>
+      <c r="C266" t="str">
+        <v>الزين</v>
+      </c>
+      <c r="D266">
+        <v>2026</v>
+      </c>
+      <c r="E266">
+        <v>200000</v>
+      </c>
+      <c r="F266" t="str">
+        <v>2026-01-23</v>
+      </c>
+      <c r="G266" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267">
+        <v>76</v>
+      </c>
+      <c r="B267" t="str">
+        <v>أميرة</v>
+      </c>
+      <c r="C267" t="str">
+        <v>العمر</v>
+      </c>
+      <c r="D267">
+        <v>2026</v>
+      </c>
+      <c r="E267">
+        <v>200000</v>
+      </c>
+      <c r="F267" t="str">
+        <v>2026-07-04</v>
+      </c>
+      <c r="G267" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268">
+        <v>77</v>
+      </c>
+      <c r="B268" t="str">
+        <v>هلا</v>
+      </c>
+      <c r="C268" t="str">
+        <v>الزين</v>
+      </c>
+      <c r="D268">
+        <v>2026</v>
+      </c>
+      <c r="E268">
+        <v>200000</v>
+      </c>
+      <c r="F268" t="str">
+        <v>2026-08-01</v>
+      </c>
+      <c r="G268" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269">
+        <v>78</v>
+      </c>
+      <c r="B269" t="str">
+        <v>هلا</v>
+      </c>
+      <c r="C269" t="str">
+        <v>الدمشقي</v>
+      </c>
+      <c r="D269">
+        <v>2026</v>
+      </c>
+      <c r="E269">
+        <v>200000</v>
+      </c>
+      <c r="F269" t="str">
+        <v>2026-06-07</v>
+      </c>
+      <c r="G269" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270">
+        <v>79</v>
+      </c>
+      <c r="B270" t="str">
+        <v>لمى</v>
+      </c>
+      <c r="C270" t="str">
+        <v>الكردي</v>
+      </c>
+      <c r="D270">
+        <v>2026</v>
+      </c>
+      <c r="E270">
+        <v>250000</v>
+      </c>
+      <c r="F270" t="str">
+        <v>2026-11-24</v>
+      </c>
+      <c r="G270" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271">
+        <v>80</v>
+      </c>
+      <c r="B271" t="str">
+        <v>نور</v>
+      </c>
+      <c r="C271" t="str">
+        <v>الدباغ</v>
+      </c>
+      <c r="D271">
+        <v>2026</v>
+      </c>
+      <c r="E271">
+        <v>200000</v>
+      </c>
+      <c r="F271" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="G271" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272">
+        <v>81</v>
+      </c>
+      <c r="B272" t="str">
+        <v>رنا</v>
+      </c>
+      <c r="C272" t="str">
+        <v>البني</v>
+      </c>
+      <c r="D272">
+        <v>2026</v>
+      </c>
+      <c r="E272">
+        <v>300000</v>
+      </c>
+      <c r="F272" t="str">
+        <v>2026-03-06</v>
+      </c>
+      <c r="G272" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273">
+        <v>82</v>
+      </c>
+      <c r="B273" t="str">
+        <v>نور</v>
+      </c>
+      <c r="C273" t="str">
+        <v>الخطيب</v>
+      </c>
+      <c r="D273">
+        <v>2026</v>
+      </c>
+      <c r="E273">
+        <v>200000</v>
+      </c>
+      <c r="F273" t="str">
+        <v>2026-09-05</v>
+      </c>
+      <c r="G273" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274">
+        <v>83</v>
+      </c>
+      <c r="B274" t="str">
+        <v>شيماء</v>
+      </c>
+      <c r="C274" t="str">
+        <v>الرفاعي</v>
+      </c>
+      <c r="D274">
+        <v>2026</v>
+      </c>
+      <c r="E274">
+        <v>200000</v>
+      </c>
+      <c r="F274" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="G274" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275">
+        <v>84</v>
+      </c>
+      <c r="B275" t="str">
+        <v>نور</v>
+      </c>
+      <c r="C275" t="str">
+        <v>الشامي</v>
+      </c>
+      <c r="D275">
+        <v>2026</v>
+      </c>
+      <c r="E275">
+        <v>200000</v>
+      </c>
+      <c r="F275" t="str">
+        <v>2026-05-18</v>
+      </c>
+      <c r="G275" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276">
+        <v>85</v>
+      </c>
+      <c r="B276" t="str">
+        <v>منى</v>
+      </c>
+      <c r="C276" t="str">
+        <v>الهاشم</v>
+      </c>
+      <c r="D276">
+        <v>2026</v>
+      </c>
+      <c r="E276">
+        <v>200000</v>
+      </c>
+      <c r="F276" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="G276" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277">
+        <v>86</v>
+      </c>
+      <c r="B277" t="str">
+        <v>أميرة</v>
+      </c>
+      <c r="C277" t="str">
+        <v>المصري</v>
+      </c>
+      <c r="D277">
+        <v>2026</v>
+      </c>
+      <c r="E277">
+        <v>250000</v>
+      </c>
+      <c r="F277" t="str">
+        <v>2026-03-04</v>
+      </c>
+      <c r="G277" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278">
+        <v>87</v>
+      </c>
+      <c r="B278" t="str">
+        <v>لمى</v>
+      </c>
+      <c r="C278" t="str">
+        <v>السيد</v>
+      </c>
+      <c r="D278">
+        <v>2026</v>
+      </c>
+      <c r="E278">
+        <v>200000</v>
+      </c>
+      <c r="F278" t="str">
+        <v>2026-11-15</v>
+      </c>
+      <c r="G278" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279">
+        <v>88</v>
+      </c>
+      <c r="B279" t="str">
+        <v>نور</v>
+      </c>
+      <c r="C279" t="str">
+        <v>المهايني</v>
+      </c>
+      <c r="D279">
+        <v>2026</v>
+      </c>
+      <c r="E279">
+        <v>300000</v>
+      </c>
+      <c r="F279" t="str">
+        <v>2026-04-22</v>
+      </c>
+      <c r="G279" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280">
+        <v>89</v>
+      </c>
+      <c r="B280" t="str">
+        <v>سمر</v>
+      </c>
+      <c r="C280" t="str">
+        <v>السليمان</v>
+      </c>
+      <c r="D280">
+        <v>2026</v>
+      </c>
+      <c r="E280">
+        <v>200000</v>
+      </c>
+      <c r="F280" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="G280" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281">
+        <v>90</v>
+      </c>
+      <c r="B281" t="str">
+        <v>رنا</v>
+      </c>
+      <c r="C281" t="str">
+        <v>الجسر</v>
+      </c>
+      <c r="D281">
+        <v>2026</v>
+      </c>
+      <c r="E281">
+        <v>200000</v>
+      </c>
+      <c r="F281" t="str">
+        <v>2026-04-28</v>
+      </c>
+      <c r="G281" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282">
+        <v>91</v>
+      </c>
+      <c r="B282" t="str">
+        <v>شيماء</v>
+      </c>
+      <c r="C282" t="str">
+        <v>البدران</v>
+      </c>
+      <c r="D282">
+        <v>2026</v>
+      </c>
+      <c r="E282">
+        <v>200000</v>
+      </c>
+      <c r="F282" t="str">
+        <v>2026-07-26</v>
+      </c>
+      <c r="G282" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283">
+        <v>92</v>
+      </c>
+      <c r="B283" t="str">
+        <v>نادية</v>
+      </c>
+      <c r="C283" t="str">
+        <v>اليوسف</v>
+      </c>
+      <c r="D283">
+        <v>2026</v>
+      </c>
+      <c r="E283">
+        <v>200000</v>
+      </c>
+      <c r="F283" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="G283" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284">
+        <v>93</v>
+      </c>
+      <c r="B284" t="str">
+        <v>أميرة</v>
+      </c>
+      <c r="C284" t="str">
+        <v>التميمي</v>
+      </c>
+      <c r="D284">
+        <v>2026</v>
+      </c>
+      <c r="E284">
+        <v>250000</v>
+      </c>
+      <c r="F284" t="str">
+        <v>2026-08-22</v>
+      </c>
+      <c r="G284" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285">
+        <v>94</v>
+      </c>
+      <c r="B285" t="str">
+        <v>هبة</v>
+      </c>
+      <c r="C285" t="str">
+        <v>الزين</v>
+      </c>
+      <c r="D285">
+        <v>2026</v>
+      </c>
+      <c r="E285">
+        <v>200000</v>
+      </c>
+      <c r="F285" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="G285" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286">
+        <v>95</v>
+      </c>
+      <c r="B286" t="str">
+        <v>منى</v>
+      </c>
+      <c r="C286" t="str">
+        <v>الكلاس</v>
+      </c>
+      <c r="D286">
+        <v>2026</v>
+      </c>
+      <c r="E286">
+        <v>300000</v>
+      </c>
+      <c r="F286" t="str">
+        <v>2026-09-13</v>
+      </c>
+      <c r="G286" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287">
+        <v>96</v>
+      </c>
+      <c r="B287" t="str">
+        <v>منى</v>
+      </c>
+      <c r="C287" t="str">
+        <v>الكردي</v>
+      </c>
+      <c r="D287">
+        <v>2026</v>
+      </c>
+      <c r="E287">
+        <v>200000</v>
+      </c>
+      <c r="F287" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="G287" t="str">
+        <v>دُفع بالتحويل البنكي</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288">
+        <v>97</v>
+      </c>
+      <c r="B288" t="str">
+        <v>سهيلة</v>
+      </c>
+      <c r="C288" t="str">
+        <v>الرفاعي</v>
+      </c>
+      <c r="D288">
+        <v>2026</v>
+      </c>
+      <c r="E288">
+        <v>200000</v>
+      </c>
+      <c r="F288" t="str">
+        <v>2026-07-28</v>
+      </c>
+      <c r="G288" t="str">
+        <v>مُسدَّد في مقر الجمعية</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289">
+        <v>98</v>
+      </c>
+      <c r="B289" t="str">
+        <v>ميس</v>
+      </c>
+      <c r="C289" t="str">
+        <v>التميمي</v>
+      </c>
+      <c r="D289">
+        <v>2026</v>
+      </c>
+      <c r="E289">
+        <v>200000</v>
+      </c>
+      <c r="F289" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="G289" t="str">
+        <v>دُفع نقداً</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290">
+        <v>99</v>
+      </c>
+      <c r="B290" t="str">
+        <v>إيمان</v>
+      </c>
+      <c r="C290" t="str">
+        <v>العاصي</v>
+      </c>
+      <c r="D290">
+        <v>2026</v>
+      </c>
+      <c r="E290">
+        <v>200000</v>
+      </c>
+      <c r="F290" t="str">
+        <v>2026-08-04</v>
+      </c>
+      <c r="G290" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G191"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G290"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>